<commit_message>
feat: add CMO executive role + fix entity seeding and UserEditModal
</commit_message>
<xml_diff>
--- a/docs/JobTitles.xlsx
+++ b/docs/JobTitles.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fangkaryuan/cwc2.0/citadel-cwc-portal/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD2210D-EB0D-4242-84CC-BE32832D196D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD8D625-AF88-0043-8294-252CE06916D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="staff listing" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'staff listing'!$A$1:$D$34</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -187,9 +190,6 @@
     <t>Managing Director- Kuching Office</t>
   </si>
   <si>
-    <t>Citadel Wealth Partner Sdn. Bhd.</t>
-  </si>
-  <si>
     <t>Emily Chow</t>
   </si>
   <si>
@@ -341,6 +341,9 @@
   </si>
   <si>
     <t>display name</t>
+  </si>
+  <si>
+    <t>Citadel Wealth Partners Sdn. Bhd.</t>
   </si>
 </sst>
 </file>
@@ -732,16 +735,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -979,214 +982,214 @@
         <v>54</v>
       </c>
       <c r="D18" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B19" t="s">
         <v>56</v>
-      </c>
-      <c r="B19" t="s">
-        <v>57</v>
       </c>
       <c r="C19" t="s">
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" t="s">
         <v>59</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>60</v>
       </c>
-      <c r="C20" t="s">
-        <v>61</v>
-      </c>
       <c r="D20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" t="s">
         <v>62</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>63</v>
       </c>
-      <c r="C21" t="s">
-        <v>64</v>
-      </c>
       <c r="D21" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" t="s">
         <v>65</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>66</v>
       </c>
-      <c r="C22" t="s">
-        <v>67</v>
-      </c>
       <c r="D22" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" t="s">
         <v>68</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>69</v>
       </c>
-      <c r="C23" t="s">
-        <v>70</v>
-      </c>
       <c r="D23" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" t="s">
         <v>71</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>72</v>
       </c>
-      <c r="C24" t="s">
-        <v>73</v>
-      </c>
       <c r="D24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="s">
         <v>74</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>75</v>
       </c>
-      <c r="C25" t="s">
-        <v>76</v>
-      </c>
       <c r="D25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" t="s">
         <v>77</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>78</v>
       </c>
-      <c r="C26" t="s">
-        <v>79</v>
-      </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
+        <v>79</v>
+      </c>
+      <c r="B27" t="s">
         <v>80</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>81</v>
       </c>
-      <c r="C27" t="s">
-        <v>82</v>
-      </c>
       <c r="D27" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" t="s">
         <v>83</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>84</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>85</v>
-      </c>
-      <c r="D28" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" t="s">
         <v>87</v>
       </c>
-      <c r="B29" t="s">
-        <v>88</v>
-      </c>
       <c r="C29" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D29" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" t="s">
         <v>89</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>90</v>
       </c>
-      <c r="C30" t="s">
-        <v>91</v>
-      </c>
       <c r="D30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" t="s">
         <v>92</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>93</v>
       </c>
-      <c r="C31" t="s">
-        <v>94</v>
-      </c>
       <c r="D31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" t="s">
         <v>95</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>96</v>
       </c>
-      <c r="C32" t="s">
-        <v>97</v>
-      </c>
       <c r="D32" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>97</v>
+      </c>
+      <c r="B33" t="s">
         <v>98</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>99</v>
-      </c>
-      <c r="C33" t="s">
-        <v>100</v>
       </c>
       <c r="D33" t="s">
         <v>4</v>
@@ -1194,19 +1197,20 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>100</v>
+      </c>
+      <c r="B34" t="s">
         <v>101</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>102</v>
       </c>
-      <c r="C34" t="s">
-        <v>103</v>
-      </c>
       <c r="D34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D34" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>